<commit_message>
Touch AB and Touch LD boards BOM Revised.
</commit_message>
<xml_diff>
--- a/Deliverables/BOM/DigiKey_BOMs/Touch_Board_AB_DigiKey.xlsx
+++ b/Deliverables/BOM/DigiKey_BOMs/Touch_Board_AB_DigiKey.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24131"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\IbrahimHyder-ReverseEngineering\Deliverables\BOM\DigiKey_BOMs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark\IbrahimHyder-ReverseEngineering\Deliverables\BOM\DigiKey_BOMs\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0A1EAB-AF01-4A2B-9B22-0165A83EF51D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SM_Bottom_Board" sheetId="1" r:id="rId1"/>
@@ -17,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">SM_Bottom_Board!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="108">
   <si>
     <t>Description</t>
   </si>
@@ -176,9 +177,6 @@
     <t>RES SMD 1K OHM 5% 1/8W 0805</t>
   </si>
   <si>
-    <t>R1, R14</t>
-  </si>
-  <si>
     <t>RES 0805</t>
   </si>
   <si>
@@ -197,9 +195,6 @@
     <t>Res SMD 100 Ohm 0.10% 1/8W 0805</t>
   </si>
   <si>
-    <t>R3, R4, R5, R6, R7, R8, R9, R10, R11, R12, R15</t>
-  </si>
-  <si>
     <t>ERA6VEB1000V</t>
   </si>
   <si>
@@ -221,18 +216,12 @@
     <t>TVFU03</t>
   </si>
   <si>
-    <t>SOT-23-6L Touch Sensors RoHS</t>
-  </si>
-  <si>
     <t>U1, U2</t>
   </si>
   <si>
     <t>SOT-23-6</t>
   </si>
   <si>
-    <t>RH6015D</t>
-  </si>
-  <si>
     <t>0.1uF</t>
   </si>
   <si>
@@ -305,9 +294,6 @@
     <t>Yageo</t>
   </si>
   <si>
-    <t>YAGEO</t>
-  </si>
-  <si>
     <t>Local supplier</t>
   </si>
   <si>
@@ -345,12 +331,33 @@
   </si>
   <si>
     <t>Custom</t>
+  </si>
+  <si>
+    <t>RH6016D</t>
+  </si>
+  <si>
+    <t>SOT-23-6 Touch Sensors RoHS</t>
+  </si>
+  <si>
+    <t>Jianfu Electronics</t>
+  </si>
+  <si>
+    <t>RONGHE Microelectronics</t>
+  </si>
+  <si>
+    <t>------------</t>
+  </si>
+  <si>
+    <t>R1, R3, R4, R5, R6, R7, R8, R10, R11, R12, R15</t>
+  </si>
+  <si>
+    <t>R9, R14</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
@@ -480,7 +487,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -631,12 +638,117 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -659,56 +771,20 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -734,9 +810,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -761,32 +834,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="44" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -810,6 +857,109 @@
     </xf>
     <xf numFmtId="44" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="12" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="44" fontId="12" fillId="4" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1090,7 +1240,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -1122,50 +1272,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:40" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
-        <v>94</v>
-      </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
-      <c r="I1" s="20"/>
-      <c r="J1" s="20"/>
-      <c r="K1" s="20"/>
-      <c r="L1" s="20"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="20"/>
-      <c r="O1" s="20"/>
-      <c r="P1" s="20"/>
-      <c r="Q1" s="20"/>
-      <c r="R1" s="20"/>
-      <c r="S1" s="20"/>
-      <c r="T1" s="20"/>
-      <c r="U1" s="21"/>
-      <c r="V1" s="19" t="s">
+      <c r="A1" s="42" t="s">
+        <v>89</v>
+      </c>
+      <c r="B1" s="43"/>
+      <c r="C1" s="43"/>
+      <c r="D1" s="43"/>
+      <c r="E1" s="43"/>
+      <c r="F1" s="43"/>
+      <c r="G1" s="43"/>
+      <c r="H1" s="43"/>
+      <c r="I1" s="43"/>
+      <c r="J1" s="43"/>
+      <c r="K1" s="43"/>
+      <c r="L1" s="43"/>
+      <c r="M1" s="43"/>
+      <c r="N1" s="43"/>
+      <c r="O1" s="43"/>
+      <c r="P1" s="43"/>
+      <c r="Q1" s="43"/>
+      <c r="R1" s="43"/>
+      <c r="S1" s="43"/>
+      <c r="T1" s="43"/>
+      <c r="U1" s="44"/>
+      <c r="V1" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="W1" s="20"/>
-      <c r="X1" s="20"/>
-      <c r="Y1" s="20"/>
-      <c r="Z1" s="20"/>
-      <c r="AA1" s="20"/>
-      <c r="AB1" s="20"/>
-      <c r="AC1" s="20"/>
-      <c r="AD1" s="20"/>
-      <c r="AE1" s="20"/>
-      <c r="AF1" s="20"/>
-      <c r="AG1" s="20"/>
-      <c r="AH1" s="20"/>
-      <c r="AI1" s="20"/>
-      <c r="AJ1" s="20"/>
-      <c r="AK1" s="20"/>
-      <c r="AL1" s="20"/>
-      <c r="AM1" s="20"/>
-      <c r="AN1" s="21"/>
+      <c r="W1" s="43"/>
+      <c r="X1" s="43"/>
+      <c r="Y1" s="43"/>
+      <c r="Z1" s="43"/>
+      <c r="AA1" s="43"/>
+      <c r="AB1" s="43"/>
+      <c r="AC1" s="43"/>
+      <c r="AD1" s="43"/>
+      <c r="AE1" s="43"/>
+      <c r="AF1" s="43"/>
+      <c r="AG1" s="43"/>
+      <c r="AH1" s="43"/>
+      <c r="AI1" s="43"/>
+      <c r="AJ1" s="43"/>
+      <c r="AK1" s="43"/>
+      <c r="AL1" s="43"/>
+      <c r="AM1" s="43"/>
+      <c r="AN1" s="44"/>
     </row>
     <row r="2" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1239,17 +1389,17 @@
       </c>
     </row>
     <row r="3" spans="1:40" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+      <c r="A3" s="78">
         <v>1</v>
       </c>
-      <c r="B3" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="C3" s="25" t="s">
+      <c r="B3" s="60" t="s">
+        <v>91</v>
+      </c>
+      <c r="C3" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="D3" s="26" t="s">
-        <v>103</v>
+      <c r="D3" s="64" t="s">
+        <v>98</v>
       </c>
       <c r="E3" s="9" t="s">
         <v>28</v>
@@ -1258,929 +1408,937 @@
         <v>29</v>
       </c>
       <c r="G3" s="9" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="I3" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="J3" s="27">
+        <v>64</v>
+      </c>
+      <c r="J3" s="15">
         <v>7</v>
       </c>
-      <c r="K3" s="28">
+      <c r="K3" s="16">
         <f>J3*5</f>
         <v>35</v>
       </c>
-      <c r="L3" s="28">
+      <c r="L3" s="16">
         <f>J3*1000</f>
         <v>7000</v>
       </c>
-      <c r="M3" s="28">
+      <c r="M3" s="16">
         <f>J3*5000</f>
         <v>35000</v>
       </c>
-      <c r="N3" s="29" t="s">
+      <c r="N3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="O3" s="30">
+      <c r="O3" s="18">
         <v>0.12</v>
       </c>
-      <c r="P3" s="31">
+      <c r="P3" s="19">
         <f>O3*J3</f>
         <v>0.84</v>
       </c>
-      <c r="Q3" s="30">
+      <c r="Q3" s="18">
         <v>8.5999999999999993E-2</v>
       </c>
-      <c r="R3" s="31">
+      <c r="R3" s="19">
         <f>Q3*K3</f>
         <v>3.01</v>
       </c>
-      <c r="S3" s="30">
+      <c r="S3" s="18">
         <v>2.0031428571428599E-2</v>
       </c>
-      <c r="T3" s="31">
+      <c r="T3" s="19">
         <f>S3*L3</f>
         <v>140.2200000000002</v>
       </c>
-      <c r="U3" s="32">
+      <c r="U3" s="20">
         <v>1.7938285714285698E-2</v>
       </c>
-      <c r="V3" s="33">
+      <c r="V3" s="21">
         <f>U3*M3</f>
         <v>627.83999999999946</v>
       </c>
-      <c r="W3" s="34"/>
+      <c r="W3" s="22"/>
     </row>
     <row r="4" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
+      <c r="A4" s="78">
         <v>2</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="35" t="s">
+      <c r="B4" s="62"/>
+      <c r="C4" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="G4" s="36" t="s">
-        <v>80</v>
-      </c>
-      <c r="H4" s="16" t="s">
-        <v>78</v>
-      </c>
-      <c r="I4" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="J4" s="37">
+      <c r="G4" s="65" t="s">
+        <v>76</v>
+      </c>
+      <c r="H4" s="66" t="s">
+        <v>74</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="J4" s="34">
         <v>2</v>
       </c>
-      <c r="K4" s="38">
+      <c r="K4" s="35">
         <f t="shared" ref="K4:K5" si="0">J4*5</f>
         <v>10</v>
       </c>
-      <c r="L4" s="38">
+      <c r="L4" s="35">
         <f>J4*1000</f>
         <v>2000</v>
       </c>
-      <c r="M4" s="38">
+      <c r="M4" s="35">
         <f>J4*5000</f>
         <v>10000</v>
       </c>
-      <c r="N4" s="39" t="s">
+      <c r="N4" s="36" t="s">
         <v>20</v>
       </c>
-      <c r="O4" s="40">
+      <c r="O4" s="37">
         <v>0.68</v>
       </c>
-      <c r="P4" s="41">
+      <c r="P4" s="38">
         <f>O4*J4</f>
         <v>1.36</v>
       </c>
-      <c r="Q4" s="40">
+      <c r="Q4" s="37">
         <v>0.48399999999999999</v>
       </c>
-      <c r="R4" s="41">
+      <c r="R4" s="38">
         <f>Q4*K4</f>
         <v>4.84</v>
       </c>
-      <c r="S4" s="40">
+      <c r="S4" s="37">
         <v>0.20058000000000001</v>
       </c>
-      <c r="T4" s="41">
+      <c r="T4" s="38">
         <f>S4*L4</f>
         <v>401.16</v>
       </c>
-      <c r="U4" s="42">
+      <c r="U4" s="39">
         <v>0.20058000000000001</v>
       </c>
-      <c r="V4" s="43">
+      <c r="V4" s="40">
         <f>U4*M4</f>
         <v>2005.8000000000002</v>
       </c>
-      <c r="W4" s="44"/>
+      <c r="W4" s="41"/>
     </row>
     <row r="5" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+      <c r="A5" s="78">
         <v>3</v>
       </c>
-      <c r="B5" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="35" t="s">
+      <c r="B5" s="47" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="48" t="s">
         <v>34</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="49" t="s">
         <v>35</v>
       </c>
-      <c r="E5" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="F5" s="6" t="s">
+      <c r="E5" s="49" t="s">
+        <v>100</v>
+      </c>
+      <c r="F5" s="49" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="H5" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" s="37">
+      <c r="G5" s="49" t="s">
+        <v>99</v>
+      </c>
+      <c r="H5" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="I5" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="J5" s="51">
         <v>1</v>
       </c>
-      <c r="K5" s="38">
+      <c r="K5" s="52">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="L5" s="38">
-        <f t="shared" ref="L5:L14" si="1">J5*1000</f>
+      <c r="L5" s="52">
+        <f t="shared" ref="L5:L13" si="1">J5*1000</f>
         <v>1000</v>
       </c>
-      <c r="M5" s="38">
-        <f t="shared" ref="M5:M14" si="2">J5*5000</f>
+      <c r="M5" s="52">
+        <f t="shared" ref="M5:M13" si="2">J5*5000</f>
         <v>5000</v>
       </c>
-      <c r="N5" s="39" t="s">
-        <v>82</v>
-      </c>
-      <c r="O5" s="40">
+      <c r="N5" s="53" t="s">
+        <v>78</v>
+      </c>
+      <c r="O5" s="54">
         <v>1.24</v>
       </c>
-      <c r="P5" s="41">
-        <f t="shared" ref="P5:P14" si="3">O5*J5</f>
+      <c r="P5" s="55">
+        <f t="shared" ref="P5:P13" si="3">O5*J5</f>
         <v>1.24</v>
       </c>
-      <c r="Q5" s="40">
+      <c r="Q5" s="54">
         <v>1.24</v>
       </c>
-      <c r="R5" s="41">
-        <f t="shared" ref="R5:R14" si="4">Q5*K5</f>
+      <c r="R5" s="55">
+        <f t="shared" ref="R5:R13" si="4">Q5*K5</f>
         <v>6.2</v>
       </c>
-      <c r="S5" s="40">
+      <c r="S5" s="54">
         <v>0.872</v>
       </c>
-      <c r="T5" s="41">
-        <f t="shared" ref="T5:T14" si="5">S5*L5</f>
+      <c r="T5" s="55">
+        <f t="shared" ref="T5:T13" si="5">S5*L5</f>
         <v>872</v>
       </c>
-      <c r="U5" s="42">
+      <c r="U5" s="56">
         <v>0.872</v>
       </c>
-      <c r="V5" s="43">
-        <f t="shared" ref="V5:V14" si="6">U5*M5</f>
+      <c r="V5" s="57">
+        <f t="shared" ref="V5:V13" si="6">U5*M5</f>
         <v>4360</v>
       </c>
-      <c r="W5" s="45" t="s">
-        <v>81</v>
+      <c r="W5" s="59" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:40" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="1">
+      <c r="A6" s="78">
         <v>4</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" s="35" t="s">
+      <c r="B6" s="47" t="s">
+        <v>93</v>
+      </c>
+      <c r="C6" s="48" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" s="49" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" s="49" t="s">
         <v>40</v>
       </c>
-      <c r="G6" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="H6" s="11" t="s">
+      <c r="G6" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="I6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="J6" s="37">
+      <c r="H6" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="I6" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="J6" s="51">
         <v>9</v>
       </c>
-      <c r="K6" s="38">
-        <f t="shared" ref="K6:K14" si="7">J6*5</f>
+      <c r="K6" s="52">
+        <f t="shared" ref="K6:K13" si="7">J6*5</f>
         <v>45</v>
       </c>
-      <c r="L6" s="38">
+      <c r="L6" s="52">
         <f t="shared" si="1"/>
         <v>9000</v>
       </c>
-      <c r="M6" s="38">
+      <c r="M6" s="52">
         <f t="shared" si="2"/>
         <v>45000</v>
       </c>
-      <c r="N6" s="39" t="s">
+      <c r="N6" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="O6" s="40">
+      <c r="O6" s="54">
         <v>0.18</v>
       </c>
-      <c r="P6" s="41">
+      <c r="P6" s="55">
         <f t="shared" si="3"/>
         <v>1.6199999999999999</v>
       </c>
-      <c r="Q6" s="40">
+      <c r="Q6" s="54">
         <v>0.18</v>
       </c>
-      <c r="R6" s="41">
+      <c r="R6" s="55">
         <f t="shared" si="4"/>
         <v>8.1</v>
       </c>
-      <c r="S6" s="40">
+      <c r="S6" s="54">
         <v>0.123</v>
       </c>
-      <c r="T6" s="41">
+      <c r="T6" s="55">
         <f t="shared" si="5"/>
         <v>1107</v>
       </c>
-      <c r="U6" s="42">
+      <c r="U6" s="56">
         <v>0.123</v>
       </c>
-      <c r="V6" s="43">
+      <c r="V6" s="57">
         <f t="shared" si="6"/>
         <v>5535</v>
       </c>
-      <c r="W6" s="44"/>
+      <c r="W6" s="58"/>
     </row>
     <row r="7" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
+      <c r="A7" s="78">
         <v>5</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="47" t="s">
+        <v>94</v>
+      </c>
+      <c r="C7" s="48" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="49" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="49" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="49" t="s">
+        <v>82</v>
+      </c>
+      <c r="H7" s="63" t="s">
+        <v>81</v>
+      </c>
+      <c r="I7" s="50" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="46" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="47" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="F7" s="47" t="s">
-        <v>43</v>
-      </c>
-      <c r="G7" s="47"/>
-      <c r="H7" s="48"/>
-      <c r="I7" s="47" t="s">
-        <v>70</v>
-      </c>
-      <c r="J7" s="49">
-        <v>4</v>
-      </c>
-      <c r="K7" s="50">
+      <c r="J7" s="51">
+        <v>1</v>
+      </c>
+      <c r="K7" s="52">
         <f t="shared" si="7"/>
-        <v>20</v>
-      </c>
-      <c r="L7" s="50">
+        <v>5</v>
+      </c>
+      <c r="L7" s="52">
         <f t="shared" si="1"/>
-        <v>4000</v>
-      </c>
-      <c r="M7" s="50">
+        <v>1000</v>
+      </c>
+      <c r="M7" s="52">
         <f t="shared" si="2"/>
-        <v>20000</v>
-      </c>
-      <c r="N7" s="39"/>
-      <c r="O7" s="51"/>
-      <c r="P7" s="52">
+        <v>5000</v>
+      </c>
+      <c r="N7" s="53" t="s">
+        <v>80</v>
+      </c>
+      <c r="O7" s="54">
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="P7" s="55">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-      <c r="Q7" s="51"/>
-      <c r="R7" s="52">
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="Q7" s="54">
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="R7" s="55">
         <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-      <c r="S7" s="51"/>
-      <c r="T7" s="52">
+        <v>1.31</v>
+      </c>
+      <c r="S7" s="54">
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="T7" s="55">
         <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-      <c r="U7" s="53"/>
-      <c r="V7" s="54">
+        <v>262</v>
+      </c>
+      <c r="U7" s="54">
+        <v>0.26200000000000001</v>
+      </c>
+      <c r="V7" s="57">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="W7" s="55" t="s">
-        <v>76</v>
-      </c>
+        <v>1310</v>
+      </c>
+      <c r="W7" s="58"/>
     </row>
     <row r="8" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1">
+      <c r="A8" s="78">
         <v>6</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>44</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="6" t="s">
+      <c r="B8" s="60" t="s">
+        <v>95</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="H8" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="J8" s="15">
+        <v>2</v>
+      </c>
+      <c r="K8" s="16">
+        <f t="shared" si="7"/>
+        <v>10</v>
+      </c>
+      <c r="L8" s="16">
+        <f t="shared" si="1"/>
+        <v>2000</v>
+      </c>
+      <c r="M8" s="16">
+        <f t="shared" si="2"/>
+        <v>10000</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="O8" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="P8" s="19">
+        <f t="shared" si="3"/>
+        <v>0.2</v>
+      </c>
+      <c r="Q8" s="18">
+        <v>0.05</v>
+      </c>
+      <c r="R8" s="19">
+        <f t="shared" si="4"/>
+        <v>0.5</v>
+      </c>
+      <c r="S8" s="18">
+        <v>9.1400000000000006E-3</v>
+      </c>
+      <c r="T8" s="19">
+        <f t="shared" si="5"/>
+        <v>18.28</v>
+      </c>
+      <c r="U8" s="20">
+        <v>6.5599999999999999E-3</v>
+      </c>
+      <c r="V8" s="21">
+        <f t="shared" si="6"/>
+        <v>65.599999999999994</v>
+      </c>
+      <c r="W8" s="22"/>
+    </row>
+    <row r="9" spans="1:40" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="78">
+        <v>7</v>
+      </c>
+      <c r="B9" s="61"/>
+      <c r="C9" s="23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="J9" s="24">
+        <v>3</v>
+      </c>
+      <c r="K9" s="25">
+        <f t="shared" si="7"/>
+        <v>15</v>
+      </c>
+      <c r="L9" s="25">
+        <f t="shared" si="1"/>
+        <v>3000</v>
+      </c>
+      <c r="M9" s="25">
+        <f t="shared" si="2"/>
+        <v>15000</v>
+      </c>
+      <c r="N9" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="O9" s="27">
+        <v>0.31</v>
+      </c>
+      <c r="P9" s="28">
+        <f t="shared" si="3"/>
+        <v>0.92999999999999994</v>
+      </c>
+      <c r="Q9" s="27">
+        <v>0.26600000000000001</v>
+      </c>
+      <c r="R9" s="28">
+        <f>(0.266*10)+(0.31*5)</f>
+        <v>4.21</v>
+      </c>
+      <c r="S9" s="27">
+        <v>3.9849999999999997E-2</v>
+      </c>
+      <c r="T9" s="28">
+        <f t="shared" si="5"/>
+        <v>119.54999999999998</v>
+      </c>
+      <c r="U9" s="29">
+        <v>3.6220000000000002E-2</v>
+      </c>
+      <c r="V9" s="30">
+        <f t="shared" si="6"/>
+        <v>543.30000000000007</v>
+      </c>
+      <c r="W9" s="31"/>
+    </row>
+    <row r="10" spans="1:40" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="78">
+        <v>8</v>
+      </c>
+      <c r="B10" s="61"/>
+      <c r="C10" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H10" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="H8" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="I8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="J8" s="37">
+      <c r="I10" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="J10" s="24">
+        <v>11</v>
+      </c>
+      <c r="K10" s="25">
+        <f t="shared" si="7"/>
+        <v>55</v>
+      </c>
+      <c r="L10" s="25">
+        <f t="shared" si="1"/>
+        <v>11000</v>
+      </c>
+      <c r="M10" s="25">
+        <f t="shared" si="2"/>
+        <v>55000</v>
+      </c>
+      <c r="N10" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="O10" s="25">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="P10" s="28">
+        <f>(O10*10)+0.1</f>
+        <v>0.52999999999999992</v>
+      </c>
+      <c r="Q10" s="25">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="R10" s="28">
+        <f>(Q10*50)+(0.1*5)</f>
+        <v>2.65</v>
+      </c>
+      <c r="S10" s="27">
+        <v>7.77E-3</v>
+      </c>
+      <c r="T10" s="28">
+        <f t="shared" si="5"/>
+        <v>85.47</v>
+      </c>
+      <c r="U10" s="29">
+        <v>5.5700000000000003E-3</v>
+      </c>
+      <c r="V10" s="30">
+        <f t="shared" si="6"/>
+        <v>306.35000000000002</v>
+      </c>
+      <c r="W10" s="32"/>
+    </row>
+    <row r="11" spans="1:40" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="78">
+        <v>9</v>
+      </c>
+      <c r="B11" s="62"/>
+      <c r="C11" s="33" t="s">
+        <v>56</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="E11" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="H11" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="I11" s="11" t="s">
+        <v>70</v>
+      </c>
+      <c r="J11" s="34">
         <v>1</v>
       </c>
-      <c r="K8" s="38">
+      <c r="K11" s="35">
         <f t="shared" si="7"/>
         <v>5</v>
       </c>
-      <c r="L8" s="38">
+      <c r="L11" s="35">
         <f t="shared" si="1"/>
         <v>1000</v>
       </c>
-      <c r="M8" s="38">
+      <c r="M11" s="35">
         <f t="shared" si="2"/>
         <v>5000</v>
       </c>
-      <c r="N8" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="O8" s="40">
-        <v>0.26200000000000001</v>
-      </c>
-      <c r="P8" s="41">
+      <c r="N11" s="36" t="s">
+        <v>80</v>
+      </c>
+      <c r="O11" s="37">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="P11" s="38">
         <f t="shared" si="3"/>
-        <v>0.26200000000000001</v>
-      </c>
-      <c r="Q8" s="40">
-        <v>0.26200000000000001</v>
-      </c>
-      <c r="R8" s="41">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="Q11" s="37">
+        <v>0.10100000000000001</v>
+      </c>
+      <c r="R11" s="38">
         <f t="shared" si="4"/>
-        <v>1.31</v>
-      </c>
-      <c r="S8" s="40">
-        <v>0.26200000000000001</v>
-      </c>
-      <c r="T8" s="41">
+        <v>0.505</v>
+      </c>
+      <c r="S11" s="37">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="T11" s="38">
         <f t="shared" si="5"/>
-        <v>262</v>
-      </c>
-      <c r="U8" s="40">
-        <v>0.26200000000000001</v>
-      </c>
-      <c r="V8" s="43">
+        <v>7</v>
+      </c>
+      <c r="U11" s="39">
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="V11" s="40">
         <f t="shared" si="6"/>
-        <v>1310</v>
-      </c>
-      <c r="W8" s="44"/>
+        <v>35</v>
+      </c>
+      <c r="W11" s="41"/>
     </row>
-    <row r="9" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1">
-        <v>7</v>
-      </c>
-      <c r="B9" s="18" t="s">
+    <row r="12" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="78">
+        <v>10</v>
+      </c>
+      <c r="B12" s="47" t="s">
+        <v>96</v>
+      </c>
+      <c r="C12" s="48" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="49" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="49" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="35" t="s">
-        <v>48</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" s="6" t="s">
+      <c r="F12" s="49" t="s">
+        <v>61</v>
+      </c>
+      <c r="G12" s="50" t="s">
+        <v>103</v>
+      </c>
+      <c r="H12" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="I12" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" s="51">
+        <v>1</v>
+      </c>
+      <c r="K12" s="52">
+        <f t="shared" si="7"/>
+        <v>5</v>
+      </c>
+      <c r="L12" s="52">
+        <f t="shared" si="1"/>
+        <v>1000</v>
+      </c>
+      <c r="M12" s="52">
+        <f t="shared" si="2"/>
+        <v>5000</v>
+      </c>
+      <c r="N12" s="53" t="s">
         <v>88</v>
       </c>
-      <c r="H9" s="11"/>
-      <c r="I9" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="J9" s="37">
+      <c r="O12" s="54">
+        <v>0.15</v>
+      </c>
+      <c r="P12" s="55">
+        <f t="shared" si="3"/>
+        <v>0.15</v>
+      </c>
+      <c r="Q12" s="54">
+        <v>0.15</v>
+      </c>
+      <c r="R12" s="55">
+        <f t="shared" si="4"/>
+        <v>0.75</v>
+      </c>
+      <c r="S12" s="54">
+        <v>0.15</v>
+      </c>
+      <c r="T12" s="55">
+        <f t="shared" si="5"/>
+        <v>150</v>
+      </c>
+      <c r="U12" s="56">
+        <v>0.1</v>
+      </c>
+      <c r="V12" s="57">
+        <f t="shared" si="6"/>
+        <v>500</v>
+      </c>
+      <c r="W12" s="59" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="13" spans="1:40" ht="27" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="78">
+        <v>11</v>
+      </c>
+      <c r="B13" s="47" t="s">
+        <v>97</v>
+      </c>
+      <c r="C13" s="48" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="49" t="s">
+        <v>62</v>
+      </c>
+      <c r="E13" s="49" t="s">
+        <v>63</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="G13" s="50" t="s">
+        <v>104</v>
+      </c>
+      <c r="H13" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="I13" s="50" t="s">
+        <v>75</v>
+      </c>
+      <c r="J13" s="51">
         <v>2</v>
       </c>
-      <c r="K9" s="38">
+      <c r="K13" s="52">
         <f t="shared" si="7"/>
         <v>10</v>
       </c>
-      <c r="L9" s="38">
+      <c r="L13" s="52">
         <f t="shared" si="1"/>
         <v>2000</v>
       </c>
-      <c r="M9" s="38">
+      <c r="M13" s="52">
         <f t="shared" si="2"/>
         <v>10000</v>
       </c>
-      <c r="N9" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="O9" s="40">
-        <v>0.1</v>
-      </c>
-      <c r="P9" s="41">
+      <c r="N13" s="53" t="s">
+        <v>88</v>
+      </c>
+      <c r="O13" s="54">
+        <v>0.65</v>
+      </c>
+      <c r="P13" s="55">
         <f t="shared" si="3"/>
-        <v>0.2</v>
-      </c>
-      <c r="Q9" s="40">
-        <v>0.05</v>
-      </c>
-      <c r="R9" s="41">
+        <v>1.3</v>
+      </c>
+      <c r="Q13" s="54">
+        <v>0.63</v>
+      </c>
+      <c r="R13" s="55">
         <f t="shared" si="4"/>
-        <v>0.5</v>
-      </c>
-      <c r="S9" s="40">
-        <v>9.1400000000000006E-3</v>
-      </c>
-      <c r="T9" s="41">
+        <v>6.3</v>
+      </c>
+      <c r="S13" s="54">
+        <v>0.56999999999999995</v>
+      </c>
+      <c r="T13" s="55">
         <f t="shared" si="5"/>
-        <v>18.28</v>
-      </c>
-      <c r="U9" s="42">
-        <v>6.5599999999999999E-3</v>
-      </c>
-      <c r="V9" s="43">
+        <v>1140</v>
+      </c>
+      <c r="U13" s="56">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="V13" s="57">
         <f t="shared" si="6"/>
-        <v>65.599999999999994</v>
-      </c>
-      <c r="W9" s="45"/>
-    </row>
-    <row r="10" spans="1:40" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1">
-        <v>8</v>
-      </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="35" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="H10" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="J10" s="37">
-        <v>3</v>
-      </c>
-      <c r="K10" s="38">
-        <f t="shared" si="7"/>
-        <v>15</v>
-      </c>
-      <c r="L10" s="38">
-        <f t="shared" si="1"/>
-        <v>3000</v>
-      </c>
-      <c r="M10" s="38">
-        <f t="shared" si="2"/>
-        <v>15000</v>
-      </c>
-      <c r="N10" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="O10" s="40">
-        <v>0.31</v>
-      </c>
-      <c r="P10" s="41">
-        <f t="shared" si="3"/>
-        <v>0.92999999999999994</v>
-      </c>
-      <c r="Q10" s="40">
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="R10" s="41">
-        <f>(0.266*10)+(0.31*5)</f>
-        <v>4.21</v>
-      </c>
-      <c r="S10" s="40">
-        <v>3.9849999999999997E-2</v>
-      </c>
-      <c r="T10" s="41">
-        <f t="shared" si="5"/>
-        <v>119.54999999999998</v>
-      </c>
-      <c r="U10" s="42">
-        <v>3.6220000000000002E-2</v>
-      </c>
-      <c r="V10" s="43">
-        <f t="shared" si="6"/>
-        <v>543.30000000000007</v>
-      </c>
-      <c r="W10" s="44"/>
-    </row>
-    <row r="11" spans="1:40" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <v>9</v>
-      </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="35" t="s">
-        <v>55</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>90</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="J11" s="37">
-        <v>11</v>
-      </c>
-      <c r="K11" s="38">
-        <f t="shared" si="7"/>
-        <v>55</v>
-      </c>
-      <c r="L11" s="38">
-        <f t="shared" si="1"/>
-        <v>11000</v>
-      </c>
-      <c r="M11" s="38">
-        <f t="shared" si="2"/>
-        <v>55000</v>
-      </c>
-      <c r="N11" s="39" t="s">
-        <v>20</v>
-      </c>
-      <c r="O11" s="38">
-        <v>4.2999999999999997E-2</v>
-      </c>
-      <c r="P11" s="41">
-        <f>(O11*10)+0.1</f>
-        <v>0.52999999999999992</v>
-      </c>
-      <c r="Q11" s="38">
-        <v>4.2999999999999997E-2</v>
-      </c>
-      <c r="R11" s="41">
-        <f>(Q11*50)+(0.1*5)</f>
-        <v>2.65</v>
-      </c>
-      <c r="S11" s="40">
-        <v>7.77E-3</v>
-      </c>
-      <c r="T11" s="41">
-        <f t="shared" si="5"/>
-        <v>85.47</v>
-      </c>
-      <c r="U11" s="42">
-        <v>5.5700000000000003E-3</v>
-      </c>
-      <c r="V11" s="43">
-        <f t="shared" si="6"/>
-        <v>306.35000000000002</v>
-      </c>
-      <c r="W11" s="45"/>
-    </row>
-    <row r="12" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="1">
-        <v>10</v>
-      </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="35" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="J12" s="37">
-        <v>1</v>
-      </c>
-      <c r="K12" s="38">
-        <f t="shared" si="7"/>
-        <v>5</v>
-      </c>
-      <c r="L12" s="38">
-        <f t="shared" si="1"/>
-        <v>1000</v>
-      </c>
-      <c r="M12" s="38">
-        <f t="shared" si="2"/>
-        <v>5000</v>
-      </c>
-      <c r="N12" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="O12" s="40">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="P12" s="41">
-        <f t="shared" si="3"/>
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="Q12" s="40">
-        <v>0.10100000000000001</v>
-      </c>
-      <c r="R12" s="41">
-        <f t="shared" si="4"/>
-        <v>0.505</v>
-      </c>
-      <c r="S12" s="40">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="T12" s="41">
-        <f t="shared" si="5"/>
-        <v>7</v>
-      </c>
-      <c r="U12" s="42">
-        <v>7.0000000000000001E-3</v>
-      </c>
-      <c r="V12" s="43">
-        <f t="shared" si="6"/>
-        <v>35</v>
-      </c>
-      <c r="W12" s="44"/>
-    </row>
-    <row r="13" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="1">
-        <v>11</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="C13" s="35" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="G13" s="6"/>
-      <c r="H13" s="11" t="s">
-        <v>79</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="J13" s="37">
-        <v>1</v>
-      </c>
-      <c r="K13" s="38">
-        <f t="shared" si="7"/>
-        <v>5</v>
-      </c>
-      <c r="L13" s="38">
-        <f t="shared" si="1"/>
-        <v>1000</v>
-      </c>
-      <c r="M13" s="38">
-        <f t="shared" si="2"/>
-        <v>5000</v>
-      </c>
-      <c r="N13" s="39" t="s">
-        <v>93</v>
-      </c>
-      <c r="O13" s="40">
-        <v>0.15</v>
-      </c>
-      <c r="P13" s="41">
-        <f t="shared" si="3"/>
-        <v>0.15</v>
-      </c>
-      <c r="Q13" s="40">
-        <v>0.15</v>
-      </c>
-      <c r="R13" s="41">
-        <f t="shared" si="4"/>
-        <v>0.75</v>
-      </c>
-      <c r="S13" s="40">
-        <v>0.15</v>
-      </c>
-      <c r="T13" s="41">
-        <f t="shared" si="5"/>
-        <v>150</v>
-      </c>
-      <c r="U13" s="42">
-        <v>0.1</v>
-      </c>
-      <c r="V13" s="43">
-        <f t="shared" si="6"/>
-        <v>500</v>
-      </c>
-      <c r="W13" s="45" t="s">
-        <v>95</v>
-      </c>
+        <v>5500</v>
+      </c>
+      <c r="W13" s="58"/>
     </row>
     <row r="14" spans="1:40" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="1">
+      <c r="A14" s="78">
         <v>12</v>
       </c>
-      <c r="B14" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C14" s="56" t="s">
-        <v>64</v>
-      </c>
-      <c r="D14" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E14" s="14" t="s">
+      <c r="B14" s="67" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14" s="68" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="69" t="s">
+        <v>42</v>
+      </c>
+      <c r="E14" s="69" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="69" t="s">
+        <v>43</v>
+      </c>
+      <c r="G14" s="69" t="s">
+        <v>105</v>
+      </c>
+      <c r="H14" s="70"/>
+      <c r="I14" s="69" t="s">
         <v>66</v>
       </c>
-      <c r="F14" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="G14" s="14"/>
-      <c r="H14" s="15" t="s">
-        <v>79</v>
-      </c>
-      <c r="I14" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="J14" s="57">
-        <v>2</v>
-      </c>
-      <c r="K14" s="58">
-        <f t="shared" si="7"/>
-        <v>10</v>
-      </c>
-      <c r="L14" s="58">
-        <f t="shared" si="1"/>
-        <v>2000</v>
-      </c>
-      <c r="M14" s="58">
-        <f t="shared" si="2"/>
-        <v>10000</v>
-      </c>
-      <c r="N14" s="59" t="s">
-        <v>93</v>
-      </c>
-      <c r="O14" s="60">
-        <v>1.25</v>
-      </c>
-      <c r="P14" s="61">
-        <f t="shared" si="3"/>
-        <v>2.5</v>
-      </c>
-      <c r="Q14" s="60">
-        <v>1.05</v>
-      </c>
-      <c r="R14" s="61">
-        <f t="shared" si="4"/>
-        <v>10.5</v>
-      </c>
-      <c r="S14" s="60">
-        <v>0.88500000000000001</v>
-      </c>
-      <c r="T14" s="61">
-        <f t="shared" si="5"/>
-        <v>1770</v>
-      </c>
-      <c r="U14" s="62">
-        <v>0.88500000000000001</v>
-      </c>
-      <c r="V14" s="63">
-        <f t="shared" si="6"/>
-        <v>8850</v>
-      </c>
-      <c r="W14" s="64"/>
+      <c r="J14" s="71">
+        <v>4</v>
+      </c>
+      <c r="K14" s="72">
+        <f>J14*5</f>
+        <v>20</v>
+      </c>
+      <c r="L14" s="72">
+        <f>J14*1000</f>
+        <v>4000</v>
+      </c>
+      <c r="M14" s="72">
+        <f>J14*5000</f>
+        <v>20000</v>
+      </c>
+      <c r="N14" s="53"/>
+      <c r="O14" s="73"/>
+      <c r="P14" s="74">
+        <f>O14*J14</f>
+        <v>0</v>
+      </c>
+      <c r="Q14" s="73"/>
+      <c r="R14" s="74">
+        <f>Q14*K14</f>
+        <v>0</v>
+      </c>
+      <c r="S14" s="73"/>
+      <c r="T14" s="74">
+        <f>S14*L14</f>
+        <v>0</v>
+      </c>
+      <c r="U14" s="75"/>
+      <c r="V14" s="76">
+        <f>U14*M14</f>
+        <v>0</v>
+      </c>
+      <c r="W14" s="77" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="15" spans="1:40" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J15" s="22" t="s">
+      <c r="J15" s="45" t="s">
         <v>17</v>
       </c>
-      <c r="K15" s="22"/>
-      <c r="L15" s="22"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="22"/>
+      <c r="K15" s="45"/>
+      <c r="L15" s="45"/>
+      <c r="M15" s="45"/>
+      <c r="N15" s="45"/>
+      <c r="O15" s="45"/>
       <c r="R15" s="3">
-        <f>SUM(R3:R14)</f>
-        <v>42.574999999999996</v>
+        <f>SUM(R3:R13)</f>
+        <v>38.374999999999993</v>
       </c>
       <c r="S15" s="3"/>
       <c r="T15" s="3">
-        <f>SUM(T3:T14)</f>
-        <v>4932.68</v>
+        <f>SUM(T3:T13)</f>
+        <v>4302.68</v>
       </c>
       <c r="V15" s="7">
-        <f>SUM(V3:V14)</f>
-        <v>24138.89</v>
+        <f>SUM(V3:V13)</f>
+        <v>20788.89</v>
       </c>
     </row>
     <row r="16" spans="1:40" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="J16" s="23" t="s">
+      <c r="J16" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="K16" s="23"/>
-      <c r="L16" s="23"/>
-      <c r="M16" s="23"/>
-      <c r="N16" s="23"/>
-      <c r="O16" s="23"/>
+      <c r="K16" s="46"/>
+      <c r="L16" s="46"/>
+      <c r="M16" s="46"/>
+      <c r="N16" s="46"/>
+      <c r="O16" s="46"/>
       <c r="P16" s="2">
-        <f>SUM(P3:P14)</f>
-        <v>9.7330000000000005</v>
+        <f>SUM(P3:P13)</f>
+        <v>8.5330000000000013</v>
       </c>
       <c r="R16" s="4">
         <f>R15/5</f>
-        <v>8.5149999999999988</v>
+        <v>7.6749999999999989</v>
       </c>
       <c r="S16" s="4"/>
       <c r="T16" s="4">
         <f>T15/1000</f>
-        <v>4.9326800000000004</v>
+        <v>4.3026800000000005</v>
       </c>
       <c r="V16" s="7">
         <f>V15/5000</f>
-        <v>4.8277779999999995</v>
+        <v>4.1577779999999995</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B9:B12"/>
+    <mergeCell ref="B8:B11"/>
     <mergeCell ref="V1:AN1"/>
     <mergeCell ref="J15:O15"/>
     <mergeCell ref="J16:O16"/>
@@ -2228,20 +2386,6 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S3:T7 S9:T14 T8">
-    <cfRule type="dataBar" priority="17">
-      <dataBar>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFF555A"/>
-      </dataBar>
-      <extLst>
-        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{BC439CAB-0450-4930-B07F-0CD52FB2A12C}</x14:id>
-        </ext>
-      </extLst>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="R3:R14">
     <cfRule type="dataBar" priority="2">
       <dataBar>
@@ -2270,16 +2414,30 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="S3:T6 T7 S8:T14">
+    <cfRule type="dataBar" priority="22">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFF555A"/>
+      </dataBar>
+      <extLst>
+        <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
+          <x14:id>{BC439CAB-0450-4930-B07F-0CD52FB2A12C}</x14:id>
+        </ext>
+      </extLst>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="N3" r:id="rId1"/>
-    <hyperlink ref="N4" r:id="rId2"/>
-    <hyperlink ref="N5" r:id="rId3" display="DigiKey"/>
-    <hyperlink ref="N6" r:id="rId4"/>
-    <hyperlink ref="N8" r:id="rId5"/>
-    <hyperlink ref="N9" r:id="rId6"/>
-    <hyperlink ref="N10" r:id="rId7"/>
-    <hyperlink ref="N11" r:id="rId8"/>
-    <hyperlink ref="N12" r:id="rId9"/>
+    <hyperlink ref="N3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="N4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="N5" r:id="rId3" display="DigiKey" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="N6" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="N7" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="N8" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="N9" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="N10" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="N11" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
   </hyperlinks>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0.30555555555555558" right="0.30555555555555558" top="0.30555555555555558" bottom="0.30555555555555558" header="0" footer="0"/>
@@ -2314,19 +2472,6 @@
           <xm:sqref>P3:P14</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{BC439CAB-0450-4930-B07F-0CD52FB2A12C}">
-            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
-              <x14:cfvo type="autoMin"/>
-              <x14:cfvo type="autoMax"/>
-              <x14:borderColor rgb="FFFF555A"/>
-              <x14:negativeFillColor rgb="FFFF0000"/>
-              <x14:negativeBorderColor rgb="FFFF0000"/>
-              <x14:axisColor rgb="FF000000"/>
-            </x14:dataBar>
-          </x14:cfRule>
-          <xm:sqref>S3:T7 S9:T14 T8</xm:sqref>
-        </x14:conditionalFormatting>
-        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="dataBar" id="{EA6B6037-A035-49C7-B24F-FF6A26E8D0C5}">
             <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
               <x14:cfvo type="autoMin"/>
@@ -2352,6 +2497,19 @@
           </x14:cfRule>
           <xm:sqref>V3:V14</xm:sqref>
         </x14:conditionalFormatting>
+        <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+          <x14:cfRule type="dataBar" id="{BC439CAB-0450-4930-B07F-0CD52FB2A12C}">
+            <x14:dataBar minLength="0" maxLength="100" border="1" negativeBarBorderColorSameAsPositive="0">
+              <x14:cfvo type="autoMin"/>
+              <x14:cfvo type="autoMax"/>
+              <x14:borderColor rgb="FFFF555A"/>
+              <x14:negativeFillColor rgb="FFFF0000"/>
+              <x14:negativeBorderColor rgb="FFFF0000"/>
+              <x14:axisColor rgb="FF000000"/>
+            </x14:dataBar>
+          </x14:cfRule>
+          <xm:sqref>S3:T6 T7 S8:T14</xm:sqref>
+        </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
   </extLst>

</xml_diff>